<commit_message>
[v1.8.0] Tabla Responsables en Resumen
</commit_message>
<xml_diff>
--- a/src/test/resources/fixtures/extraccion.xlsx
+++ b/src/test/resources/fixtures/extraccion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1767,83 +1767,158 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P-015</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Regresion responsable MAYUS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TRESP1@x</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>20</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Obj V</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>CTR-100</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>M-1009</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>